<commit_message>
Ready to fit rest
</commit_message>
<xml_diff>
--- a/BeatnotePostHotCell/AllFits.xlsx
+++ b/BeatnotePostHotCell/AllFits.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Diego\git\6s7p\BeatnotePostHotCell\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38A6EFC5-3829-434D-A8A4-E6ACC2BD1273}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -14,12 +20,194 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="58">
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>May22,2026+11-50-22AM</t>
+  </si>
+  <si>
+    <t>May22,2026+12-00-00PM</t>
+  </si>
+  <si>
+    <t>May22,2026+12-08-18PM</t>
+  </si>
+  <si>
+    <t>May22,2026+12-25-23PM</t>
+  </si>
+  <si>
+    <t>May22,2026+12-45-18PM</t>
+  </si>
+  <si>
+    <t>May28,2026+1-37-31PM</t>
+  </si>
+  <si>
+    <t>May28,2026+2-22-26PM</t>
+  </si>
+  <si>
+    <t>May28,2026+2-31-05PM</t>
+  </si>
+  <si>
+    <t>May28,2026+2-39-02PM</t>
+  </si>
+  <si>
+    <t>May28,2026+2-47-24PM</t>
+  </si>
+  <si>
+    <t>May28,2026+2-55-44PM</t>
+  </si>
+  <si>
+    <t>May28,2026+3-03-49PM</t>
+  </si>
+  <si>
+    <t>May28,2026+3-11-47PM</t>
+  </si>
+  <si>
+    <t>May28,2026+3-19-54PM</t>
+  </si>
+  <si>
+    <t>May28,2026+3-27-49PM</t>
+  </si>
+  <si>
+    <t>May28,2026+3-37-09PM</t>
+  </si>
+  <si>
+    <t>May28,2026+3-59-05PM</t>
+  </si>
+  <si>
+    <t>May28,2026+4-16-31PM</t>
+  </si>
+  <si>
+    <t>May28,2026+4-36-20PM</t>
+  </si>
+  <si>
+    <t>May28,2026+5-15-31PM</t>
+  </si>
+  <si>
+    <t>May28,2026+5-23-41PM</t>
+  </si>
+  <si>
+    <t>May28,2026+5-39-46PM</t>
+  </si>
+  <si>
+    <t>May28,2026+6-01-12PM</t>
+  </si>
+  <si>
+    <t>May29,2026+1-00-13PM</t>
+  </si>
+  <si>
+    <t>May29,2026+1-08-21PM</t>
+  </si>
+  <si>
+    <t>May29,2026+1-17-14PM</t>
+  </si>
+  <si>
+    <t>May29,2026+11-55-54AM</t>
+  </si>
+  <si>
+    <t>May29,2026+12-09-19PM</t>
+  </si>
+  <si>
+    <t>May29,2026+12-40-32PM</t>
+  </si>
+  <si>
+    <t>May29,2026+12-51-01PM</t>
+  </si>
+  <si>
+    <t>Jun05,2026+1-36-43PM</t>
+  </si>
+  <si>
+    <t>Jun05,2026+1-45-43PM</t>
+  </si>
+  <si>
+    <t>Jun05,2026+10-28-33AM</t>
+  </si>
+  <si>
+    <t>Jun05,2026+2-39-46PM</t>
+  </si>
+  <si>
+    <t>Jun05,2026+3-03-33PM</t>
+  </si>
+  <si>
+    <t>Jun09,2026+1-59-04PM</t>
+  </si>
+  <si>
+    <t>Jun09,2026+10-32-02AM</t>
+  </si>
+  <si>
+    <t>Jun09,2026+10-48-06AM</t>
+  </si>
+  <si>
+    <t>Jun09,2026+10-56-09AM</t>
+  </si>
+  <si>
+    <t>Jun09,2026+12-12-21PM</t>
+  </si>
+  <si>
+    <t>Jun09,2026+12-20-27PM</t>
+  </si>
+  <si>
+    <t>Jun09,2026+12-48-44PM</t>
+  </si>
+  <si>
+    <t>Jun09,2026+2-08-48PM</t>
+  </si>
+  <si>
+    <t>Jun09,2026+2-17-48PM</t>
+  </si>
+  <si>
+    <t>Jun09,2026+2-47-59PM</t>
+  </si>
+  <si>
+    <t>Jun09,2026+3-22-06PM</t>
+  </si>
+  <si>
+    <t>Jun09,2026+3-34-26PM</t>
+  </si>
+  <si>
+    <t>Jun09,2026+3-42-47PM</t>
+  </si>
+  <si>
+    <t>Jun09,2026+3-50-56PM</t>
+  </si>
+  <si>
+    <t>Jun09,2026+3-59-03PM</t>
+  </si>
+  <si>
+    <t>Jun09,2026+4-24-06PM</t>
+  </si>
+  <si>
+    <t>Jun09,2026+4-53-40PM</t>
+  </si>
+  <si>
+    <t>Jun09,2026+9-40-40AM</t>
+  </si>
+  <si>
+    <t>Jun09,2026+9-50-07AM</t>
+  </si>
+  <si>
+    <t>Jun09,2026+9-59-39AM</t>
+  </si>
+  <si>
+    <t>Alpha 456</t>
+  </si>
+  <si>
+    <t>Alpha 894</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -49,8 +237,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -330,10 +521,630 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:O56"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
+    </row>
+    <row r="2" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1">
+        <v>8.1314875900026795</v>
+      </c>
+      <c r="C2" s="1">
+        <v>0.17068222085432</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1">
+        <v>8.2055994032900799</v>
+      </c>
+      <c r="C3" s="1">
+        <v>0.169252380360598</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1">
+        <v>8.2176590050244904</v>
+      </c>
+      <c r="C4" s="1">
+        <v>0.17600556016018701</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1">
+        <v>8.2690216688035498</v>
+      </c>
+      <c r="C5" s="1">
+        <v>0.17477778117201601</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1">
+        <v>8.2739805096279504</v>
+      </c>
+      <c r="C6" s="1">
+        <v>0.17496986858800301</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="1">
+        <v>18.481531830496198</v>
+      </c>
+      <c r="C7" s="1">
+        <v>0.39075425090921301</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="1">
+        <v>18.346083770183299</v>
+      </c>
+      <c r="C8" s="1">
+        <v>0.39090251610402299</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="1">
+        <v>18.452491695077299</v>
+      </c>
+      <c r="C9" s="1">
+        <v>0.38163793874347302</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="1">
+        <v>18.351915434355199</v>
+      </c>
+      <c r="C10" s="1">
+        <v>0.38646897393750201</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="1">
+        <v>18.337397032620899</v>
+      </c>
+      <c r="C11" s="1">
+        <v>0.38820632020412599</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" s="1">
+        <v>18.232394257417202</v>
+      </c>
+      <c r="C12" s="1">
+        <v>0.391100077546855</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="1">
+        <v>18.415074041865601</v>
+      </c>
+      <c r="C13" s="1">
+        <v>0.37812534333091802</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" s="1">
+        <v>18.341941017083698</v>
+      </c>
+      <c r="C14" s="1">
+        <v>0.38449528426413199</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" s="1">
+        <v>18.237027996635099</v>
+      </c>
+      <c r="C15" s="1">
+        <v>0.38779470041263903</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16" s="1">
+        <v>18.531243546545401</v>
+      </c>
+      <c r="C16" s="1">
+        <v>0.378248054436716</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B17" s="1">
+        <v>18.412716855394802</v>
+      </c>
+      <c r="C17" s="1">
+        <v>0.388322173460803</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B18" s="1">
+        <v>18.4923898758226</v>
+      </c>
+      <c r="C18" s="1">
+        <v>0.38881861759339797</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19" s="1">
+        <v>18.515382021503999</v>
+      </c>
+      <c r="C19" s="1">
+        <v>0.39254780032303299</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B20" s="1">
+        <v>18.391192672959299</v>
+      </c>
+      <c r="C20" s="1">
+        <v>0.38860291038577099</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21" s="1">
+        <v>18.551612310419799</v>
+      </c>
+      <c r="C21" s="1">
+        <v>0.391344107724999</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B22" s="1">
+        <v>18.393990200449998</v>
+      </c>
+      <c r="C22" s="1">
+        <v>0.39401793952400199</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B23" s="1">
+        <v>18.450034969079201</v>
+      </c>
+      <c r="C23" s="1">
+        <v>0.398157579716993</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B24" s="1">
+        <v>18.408277105199002</v>
+      </c>
+      <c r="C24" s="1">
+        <v>0.38710256673105198</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B25" s="1">
+        <v>8.5185527459719204</v>
+      </c>
+      <c r="C25" s="1">
+        <v>0.18265936593662399</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B26" s="1">
+        <v>8.5260980793629599</v>
+      </c>
+      <c r="C26" s="1">
+        <v>0.17720413354468001</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B27" s="1">
+        <v>8.4894844505278897</v>
+      </c>
+      <c r="C27" s="1">
+        <v>0.183642067498062</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B28" s="1">
+        <v>8.5701060942568006</v>
+      </c>
+      <c r="C28" s="1">
+        <v>0.18126642652018499</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B29" s="1">
+        <v>8.5447049809269604</v>
+      </c>
+      <c r="C29" s="1">
+        <v>0.17863631678412401</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A30" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B30" s="1">
+        <v>8.4017872832855591</v>
+      </c>
+      <c r="C30" s="1">
+        <v>0.18200369359492499</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B31" s="1">
+        <v>8.4035403242380404</v>
+      </c>
+      <c r="C31" s="1">
+        <v>0.18140063454570701</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B32" s="1">
+        <v>8.5895120122534792</v>
+      </c>
+      <c r="C32" s="1">
+        <v>0.14198189433295499</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A33" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B33" s="1">
+        <v>8.6524212475503699</v>
+      </c>
+      <c r="C33" s="1">
+        <v>0.14200693706074399</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A34" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B34" s="1">
+        <v>8.2927304597387206</v>
+      </c>
+      <c r="C34" s="1">
+        <v>0.13879302222888601</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A35" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B35" s="1">
+        <v>8.4368095561837997</v>
+      </c>
+      <c r="C35" s="1">
+        <v>0.14134057599559999</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A36" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B36" s="1">
+        <v>8.6554109919161206</v>
+      </c>
+      <c r="C36" s="1">
+        <v>0.14287369952523299</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A37" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B37" s="1">
+        <v>8.53551089338964</v>
+      </c>
+      <c r="C37" s="1">
+        <v>0.14242039757473199</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A38" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B38" s="1">
+        <v>8.2121360213246692</v>
+      </c>
+      <c r="C38" s="1">
+        <v>0.13513280226965799</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A39" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B39" s="1">
+        <v>8.3727208112640206</v>
+      </c>
+      <c r="C39" s="1">
+        <v>0.13504563445130599</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A40" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B40" s="1">
+        <v>8.4364141305933895</v>
+      </c>
+      <c r="C40" s="1">
+        <v>0.13859780418944301</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A41" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B41" s="1">
+        <v>8.4084015562695207</v>
+      </c>
+      <c r="C41" s="1">
+        <v>0.13768382280778599</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A42" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B42" s="1">
+        <v>8.5099572412062301</v>
+      </c>
+      <c r="C42" s="1">
+        <v>0.137341027012235</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A43" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B43" s="1">
+        <v>8.4321434520724008</v>
+      </c>
+      <c r="C43" s="1">
+        <v>0.14146322755453</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A44" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B44" s="1">
+        <v>8.4721216638779193</v>
+      </c>
+      <c r="C44" s="1">
+        <v>0.1440878295095</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A45" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B45" s="1">
+        <v>8.4953666075608503</v>
+      </c>
+      <c r="C45" s="1">
+        <v>0.139203017324112</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A46" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B46" s="1">
+        <v>8.7711252103094601</v>
+      </c>
+      <c r="C46" s="1">
+        <v>0.14444988833485001</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A47" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B47" s="1">
+        <v>8.5801266895029205</v>
+      </c>
+      <c r="C47" s="1">
+        <v>0.14486186097849299</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A48" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B48" s="1">
+        <v>8.5783681642005494</v>
+      </c>
+      <c r="C48" s="1">
+        <v>0.14493175120103199</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A49" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B49" s="1">
+        <v>8.6129268121772302</v>
+      </c>
+      <c r="C49" s="1">
+        <v>0.14335784354365599</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A50" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B50" s="1">
+        <v>8.6349505815443095</v>
+      </c>
+      <c r="C50" s="1">
+        <v>0.14372426788936199</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A51" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B51" s="1">
+        <v>8.5827352500219707</v>
+      </c>
+      <c r="C51" s="1">
+        <v>0.140914458888726</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A52" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B52" s="1">
+        <v>8.6784045244654298</v>
+      </c>
+      <c r="C52" s="1">
+        <v>0.144559929539015</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A53" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B53" s="1">
+        <v>8.5889121451567796</v>
+      </c>
+      <c r="C53" s="1">
+        <v>0.13911305366694399</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A54" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B54" s="1">
+        <v>8.2237273067390202</v>
+      </c>
+      <c r="C54" s="1">
+        <v>0.136881983671574</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A55" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B55" s="1">
+        <v>8.26640584418465</v>
+      </c>
+      <c r="C55" s="1">
+        <v>0.135891683439223</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A56" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B56" s="1">
+        <v>8.2614937671479094</v>
+      </c>
+      <c r="C56" s="1">
+        <v>0.134600217130598</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>